<commit_message>
docs(sem04): corregir ortografia de Vasquez, codificacion utf-8 y alinear excel y word
</commit_message>
<xml_diff>
--- a/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
+++ b/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
@@ -123,7 +123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -277,11 +277,88 @@
         <color rgb="000F172A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00334155"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00334155"/>
+      </left>
+      <right style="thin">
+        <color rgb="00334155"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00334155"/>
+      </left>
+      <right style="thin">
+        <color rgb="00334155"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="000F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -338,6 +415,9 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -727,6 +807,7 @@
     <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="9" t="inlineStr">
         <is>
@@ -735,12 +816,12 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Implementación de un sistema web transaccional con módulos de inteligencia de negocios e inteligencia artificial para la optimización de los procesos operativos en la empresa Impresos Trujillo E.I.R.L.</t>
-        </is>
-      </c>
-      <c r="D2" s="11" t="n"/>
-      <c r="E2" s="11" t="n"/>
-      <c r="F2" s="11" t="n"/>
+          <t>Im²plem²entación de un sistem²a web transaccional con m²ódulos de inteligencia de negocios e inteligencia artificial para la optim²ización de los procesos operativos en la em²presa Im²presos Trujillo E.I.R.L.</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="22" t="n"/>
+      <c r="F2" s="23" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="9" t="inlineStr">
@@ -750,12 +831,12 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Semana 4 (Sprint 1: 14/09/2026 al 19/09/2026) | Entorno: Desarrollo Local en Docker (Sin despliegue en esta fase; VPS particular en semana 11)</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="n"/>
-      <c r="E3" s="11" t="n"/>
-      <c r="F3" s="11" t="n"/>
+          <t>Sem²ana 4 (Sprint 1: 14/09/2026 al 19/09/2026) | Entorno: Desarrollo Local en Docker (Sin despliegue en estáa fase; VPS particular en sem²ana 11)</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="n"/>
+      <c r="E3" s="22" t="n"/>
+      <c r="F3" s="23" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="13" t="inlineStr">
@@ -785,11 +866,11 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="14" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
     </row>
     <row r="6" ht="94" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
@@ -800,23 +881,23 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>• [T-03] Configuración de Docker Compose para entorno local (Angular 21 + FastAPI + PostgreSQL nativo). (Gerardo)
-• [T-04] Modelamiento de tablas relacionales de Usuarios y Roles en PostgreSQL Docker. (Diego)
-• [T-05] Maquetación inicial de estructura HTML/CSS de Login y formulario reactivo en Angular 21. (Estibb)
-• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
-• [T-07] Maquetación de componente de Login y validaciones de interfaz en Angular 21. (Estibb)
-• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)</t>
+          <t>• [T-03] Configuración de Docker Com²pose para entorno local (Angular 21 + FastAPI + PostgreSQL nativo). (Gerardo)
+• [T-04] Modelam²iento de tablas relacionales de Usuarios y Roles en PostgreSQL Docker. (Diego)
+• [T-05] Maquetación inicial de estáructura HTML/CSS de Login y form²ulario reactivo en Angular 21. (Estibb)
+• [T-06] Im²plem²entación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
+• [T-07] Maquetación de com²ponente de Login y validíaciones de interfaz en Angular 21. (Estibb)
+• [T-08] Param²etrización de catálogo de insum²os y recetas por m²² en base de díatos PostgreSQL. (Diego)</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>Sin impedimentos operativos en el primer día de sprint.</t>
+          <t>Sin im²pedim²entos operativos en el prim²er día de sprint.</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
           <t>• [T-01] Sprint Planning 1: Desglose de historias de usuario (HU-01, HU-02) en tareas técnicas. (Gerardo, Estibb, Diego)
-• [T-02] Inicialización de repositorio GitHub y configuración de ramas (main, develop). (Gerardo)</t>
+• [T-02] Inicialización de repositorio GitHub y configuración de ram²as (m²ain, develop). (Gerardo)</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
@@ -834,28 +915,28 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
-• [T-07] Maquetación de componente de Login y validaciones en Angular 21. (Estibb)
-• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)
+          <t>• [T-06] Im²plem²entación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
+• [T-07] Maquetación de com²ponente de Login y validíaciones en Angular 21. (Estibb)
+• [T-08] Param²etrización de catálogo de insum²os y recetas por m²² en base de díatos PostgreSQL. (Diego)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>Sin impedimentos activos.</t>
+          <t>Sin im²pedim²entos activos.</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>• [T-03] Configuración de Docker Compose para entorno local unificado (FastAPI, PostgreSQL, Angular). (Gerardo)
-• [T-04] Modelamiento y creación de tablas relacionales de Usuarios y Roles en PostgreSQL. (Diego)
-• [T-05] Maquetación inicial de estructura HTML/CSS de Login en Angular 21. (Estibb)</t>
+          <t>• [T-03] Configuración de Docker Com²pose para entorno local unificado (FastAPI, PostgreSQL, Angular). (Gerardo)
+• [T-04] Modelam²iento y creación de tablas relacionales de Usuarios y Roles en PostgreSQL. (Diego)
+• [T-05] Maquetación inicial de estáructura HTML/CSS de Login en Angular 21. (Estibb)</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>• [T-01] Sprint Planning 1: Desglose de HU-01 y HU-02 formalizado en el Product Backlog. (Equipo)
-• [T-02] Repositorio GitHub configurado con reglas de protección de rama main. (Gerardo)</t>
+          <t>• [T-01] Sprint Planning 1: Desglose de HU-01 y HU-02 form²alizado en el Product Backlog. (Equipo)
+• [T-02] Repositorio GitHub configurado con reglas de protección de ram²a m²ain. (Gerardo)</t>
         </is>
       </c>
     </row>
@@ -868,27 +949,27 @@
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)
+          <t>• [T-08] Param²etrización de catálogo de insum²os y recetas por m²² en base de díatos PostgreSQL. (Diego)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)
-• [T-10] Pruebas unitarias de endpoints de autenticación con pytest. (Diego)</t>
+• [T-10] Pruebas unitarias de endpoints de autenticación con pytestá. (Diego)</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>• [T-07] Esperando culminación del endpoint REST /api/v1/auth/login para integración HTTP directa en Angular. (Estibb)</t>
+          <t>• [T-07] Esperando culm²inación del endpoint REST /api/v1/auth/login para integración HTTP directa en Angular. (Estibb)</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>• [T-06] Implementación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
-• [T-07] Maquetación de vista de Login con estilos Tailwind CSS y validación de campos. (Estibb)</t>
+          <t>• [T-06] Im²plem²entación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
+• [T-07] Maquetación de vista de Login con estáilos estilos CSS nativos y validíación de cam²pos. (Estibb)</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>• [T-03] Entorno Docker local completamente operativo para todo el equipo. (Gerardo)
-• [T-04] Esquema relacional de tablas de Usuarios y Roles aplicado en PostgreSQL Docker local. (Diego)
-• [T-05] Estructura visual de componentes de Login aprobada por el equipo. (Estibb)</t>
+          <t>• [T-03] Entorno Docker local com²pletam²ente operativo para todo el equipo. (Gerardo)
+• [T-04] Esquem²a relacional de tablas de Usuarios y Roles aplicado en PostgreSQL Docker local. (Diego)
+• [T-05] Estructura visual de com²ponentes de Login aprobadía por el equipo. (Estibb)</t>
         </is>
       </c>
     </row>
@@ -901,20 +982,20 @@
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>• [T-10] Pruebas unitarias de endpoints de autenticación con pytest. (Diego)
-• [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas automatizadas locales. (Gerardo)
-• [T-12] Pruebas unitarias de componentes en Angular con Jasmine/Karma. (Estibb)</t>
+          <t>• [T-10] Pruebas unitarias de endpoints de autenticación con pytestá. (Diego)
+• [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas autom²atizadías locales. (Gerardo)
+• [T-12] Pruebas unitarias de com²ponentes en Angular con Jasm²ine/Karm²a. (Estibb)</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Sin bloqueos (Impedimento de T-07 resuelto con la publicación del endpoint de login).</t>
+          <t>Sin bloqueos (Im²pedim²ento de T-07 resuelto con la publicación del endpoint de login).</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>• [T-07] Integración del formulario de Login con API REST y gestión de tokens JWT en LocalStorage. (Estibb)
-• [T-08] Parametrización de catálogo de insumos y fórmulas de consumo por m² (HU-02). (Diego)
+          <t>• [T-07] Integración del form²ulario de Login con API REST y gestáión de tokens JWT en LocalStorage. (Estibb)
+• [T-08] Param²etrización de catálogo de insum²os y fórm²ulas de consum²o por m²² (HU-02). (Diego)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)</t>
         </is>
       </c>
@@ -933,26 +1014,26 @@
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>• [T-13] Pruebas de integración de servicios y validación de contenedores Docker en desarrollo local. (Gerardo)
-• [T-14] Demostración funcional interna del incremento de software (Sprint Review interna). (Equipo)</t>
+          <t>• [T-13] Pruebas de integración de servicios y validíación de contenedores Docker en desarrollo local. (Gerardo)
+• [T-14] Dem²ostración funcional interna del increm²ento de software (Sprint Review interna). (Equipo)</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>Sin impedimentos.</t>
+          <t>Sin im²pedim²entos.</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>• [T-10] Pruebas unitarias de endpoints con pytest y verificación de cobertura de código. (Diego)
+          <t>• [T-10] Pruebas unitarias de endpoints con pytestá y verificación de cobertura de código. (Diego)
 • [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas de integración. (Gerardo)
-• [T-12] Pruebas unitarias de componentes en Angular con Jasmine/Karma. (Estibb)</t>
+• [T-12] Pruebas unitarias de com²ponentes en Angular con Jasm²ine/Karm²a. (Estibb)</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>• [T-07] Componente de Login interactivo en Angular 21 consumiendo API REST con éxito. (Estibb)
-• [T-08] Parametrización de recetas de insumos por m² (vinilo, lona, tinta) culminada en PostgreSQL. (Diego)
+          <t>• [T-07] Com²ponente de Login interactivo en Angular 21 consum²iendo API REST con ééxito. (Estibb)
+• [T-08] Param²etrización de recetas de insum²os por m²² (vinilo, lona, tinta) culm²inadía en PostgreSQL. (Diego)
 • [T-09] Guards de navegación por roles activos en Angular 21 (bloqueo efectivo a no autorizados). (Estibb)</t>
         </is>
       </c>
@@ -966,17 +1047,17 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>• [T-15] Backlog Refinement y preparación de tareas para Sprint 2 (Cotizador y Talonario Digital HU-03, HU-04). (Equipo)</t>
+          <t>• [T-15] Backlog Refinem²ent y preparación de tareas para Sprint 2 (Cotizador y Talonario Digital HU-03, HU-04). (Equipo)</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Cero impedimentos al cierre de la semana (Despliegue a servidor VPS particular planificado para semana 11).</t>
+          <t>Cero im²pedim²entos al cierre de la sem²ana (Despliegue a servidor VPS particular planificado para sem²ana 11).</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>• [T-14] Demostración funcional interna del incremento y verificación de Definition of Done (DoD). (Gerardo, Estibb, Diego)</t>
+          <t>• [T-14] Dem²ostración funcional interna del increm²ento y verificación de Definition of Done (DoD). (Gerardo, Estibb, Diego)</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
@@ -988,12 +1069,12 @@
 • [T-05] Maquetación de interfaz de Login en Angular 21. (Estibb)
 • [T-06] API de Autenticación JWT en FastAPI. (Diego)
 • [T-07] Login frontend interactivo en Angular 21. (Estibb)
-• [T-08] Recetas de insumos por m² parametrizadas en PostgreSQL. (Diego)
+• [T-08] Recetas de insum²os por m²² param²etrizadías en PostgreSQL. (Diego)
 • [T-09] Guards de navegación RBAC en Angular 21. (Estibb)
-• [T-10] Suite de pruebas unitarias pytest (cobertura 84%). (Diego)
+• [T-10] Suite de pruebas unitarias pytestá (cobertura 84%). (Diego)
 • [T-11] Pipeline CI/CD en GitHub Actions para pruebas locales. (Gerardo)
-• [T-12] Pruebas unitarias frontend con Jasmine/Karma. (Estibb)
-• [T-13] Integración completa de servicios locales y verificación en Docker. (Gerardo)</t>
+• [T-12] Pruebas unitarias frontend con Jasm²ine/Karm²a. (Estibb)
+• [T-13] Integración com²pleta de servicios locales y verificación en Docker. (Gerardo)</t>
         </is>
       </c>
     </row>
@@ -1013,16 +1094,16 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>Total Planificadas: 15 tareas técnicas
+          <t>Total Planificadías: 15 tareas técnicas
 Historias cubiertas: HU-01 y base HU-02
 Entorno: 100% Desarrollo Local en Docker</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Impedimentos: 1 registrado (T-07)
-Estado de impedimentos: 100% resuelto
-Despliegue: Sin despliegue (VPS en semana 11)</t>
+          <t>Im²pedim²entos: 1 registrado (T-07)
+Estado de im²pedim²entos: 100% resuelto
+Despliegue: Sin despliegue (VPS en sem²ana 11)</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
@@ -1034,10 +1115,10 @@
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>Completadas al 100%: 13 tareas
-Porcentaje de Éxito de Sprint 1: 86.7%
-Story Points completados: 8 SP
-Estado: Conforme para Sprint Review</t>
+          <t>Com²pletadías al 100%: 13 tareas
+Porcentaje de Ééxito de Sprint 1: 86.7%
+Story Points com²pletados: 8 SP
+Estado: Conform²e para Sprint Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(docs): subsanar reemplazo espurio de m2 en textos y normalizar Vasquez y ortografia
</commit_message>
<xml_diff>
--- a/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
+++ b/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Im²plem²entación de un sistem²a web transaccional con m²ódulos de inteligencia de negocios e inteligencia artificial para la optim²ización de los procesos operativos en la em²presa Im²presos Trujillo E.I.R.L.</t>
+          <t>Implementación de un sistema web transaccional con módulos de inteligencia de negocios e inteligencia artificial para la optimización de los procesos operativos en la empresa Impresos Trujillo E.I.R.L.</t>
         </is>
       </c>
       <c r="D2" s="22" t="n"/>
@@ -831,7 +831,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Sem²ana 4 (Sprint 1: 14/09/2026 al 19/09/2026) | Entorno: Desarrollo Local en Docker (Sin despliegue en estáa fase; VPS particular en sem²ana 11)</t>
+          <t>Semana 4 (Sprint 1: 14/09/2026 al 19/09/2026) | Entorno: Desarrollo Local en Docker (Sin despliegue en esta fase; VPS particular en semana 11)</t>
         </is>
       </c>
       <c r="D3" s="22" t="n"/>
@@ -875,29 +875,29 @@
     <row r="6" ht="94" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 — Día 1
+          <t>Sprint 1 —— Día 1
 (Lunes 14/09/2026)</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>• [T-03] Configuración de Docker Com²pose para entorno local (Angular 21 + FastAPI + PostgreSQL nativo). (Gerardo)
-• [T-04] Modelam²iento de tablas relacionales de Usuarios y Roles en PostgreSQL Docker. (Diego)
-• [T-05] Maquetación inicial de estáructura HTML/CSS de Login y form²ulario reactivo en Angular 21. (Estibb)
-• [T-06] Im²plem²entación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
-• [T-07] Maquetación de com²ponente de Login y validíaciones de interfaz en Angular 21. (Estibb)
-• [T-08] Param²etrización de catálogo de insum²os y recetas por m²² en base de díatos PostgreSQL. (Diego)</t>
+          <t>• [T-03] Configuración de Docker Compose para entorno local (Angular 21 + FastAPI + PostgreSQL nativo). (Gerardo)
+• [T-04] Modelamiento de tablas relacionales de Usuarios y Roles en PostgreSQL Docker. (Diego)
+• [T-05] Maquetación inicial de estructura HTML/CSS de Login y formulario reactivo en Angular 21. (Estibb)
+• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
+• [T-07] Maquetación de componente de Login y validaciones de interfaz en Angular 21. (Estibb)
+• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>Sin im²pedim²entos operativos en el prim²er día de sprint.</t>
+          <t>Sin impedimentos operativos en el primer día de sprint.</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
           <t>• [T-01] Sprint Planning 1: Desglose de historias de usuario (HU-01, HU-02) en tareas técnicas. (Gerardo, Estibb, Diego)
-• [T-02] Inicialización de repositorio GitHub y configuración de ram²as (m²ain, develop). (Gerardo)</t>
+• [T-02] Inicialización de repositorio GitHub y configuración de ramas (main, develop). (Gerardo)</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
@@ -909,93 +909,93 @@
     <row r="7" ht="70" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 — Día 2
+          <t>Sprint 1 —— Día 2
 (Martes 15/09/2026)</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>• [T-06] Im²plem²entación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
-• [T-07] Maquetación de com²ponente de Login y validíaciones en Angular 21. (Estibb)
-• [T-08] Param²etrización de catálogo de insum²os y recetas por m²² en base de díatos PostgreSQL. (Diego)
+          <t>• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
+• [T-07] Maquetación de componente de Login y validaciones en Angular 21. (Estibb)
+• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>Sin im²pedim²entos activos.</t>
+          <t>Sin impedimentos activos.</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>• [T-03] Configuración de Docker Com²pose para entorno local unificado (FastAPI, PostgreSQL, Angular). (Gerardo)
-• [T-04] Modelam²iento y creación de tablas relacionales de Usuarios y Roles en PostgreSQL. (Diego)
-• [T-05] Maquetación inicial de estáructura HTML/CSS de Login en Angular 21. (Estibb)</t>
+          <t>• [T-03] Configuración de Docker Compose para entorno local unificado (FastAPI, PostgreSQL, Angular). (Gerardo)
+• [T-04] Modelamiento y creación de tablas relacionales de Usuarios y Roles en PostgreSQL. (Diego)
+• [T-05] Maquetación inicial de estructura HTML/CSS de Login en Angular 21. (Estibb)</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>• [T-01] Sprint Planning 1: Desglose de HU-01 y HU-02 form²alizado en el Product Backlog. (Equipo)
-• [T-02] Repositorio GitHub configurado con reglas de protección de ram²a m²ain. (Gerardo)</t>
+          <t>• [T-01] Sprint Planning 1: Desglose de HU-01 y HU-02 formalizado en el Product Backlog. (Equipo)
+• [T-02] Repositorio GitHub configurado con reglas de protección de rama main. (Gerardo)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 — Día 3
+          <t>Sprint 1 —— Día 3
 (Miércoles 16/09/2026)</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>• [T-08] Param²etrización de catálogo de insum²os y recetas por m²² en base de díatos PostgreSQL. (Diego)
+          <t>• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)
-• [T-10] Pruebas unitarias de endpoints de autenticación con pytestá. (Diego)</t>
+• [T-10] Pruebas unitarias de endpoints de autenticación con pytest. (Diego)</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>• [T-07] Esperando culm²inación del endpoint REST /api/v1/auth/login para integración HTTP directa en Angular. (Estibb)</t>
+          <t>• [T-07] Esperando culminación del endpoint REST /api/v1/auth/login para integración HTTP directa en Angular. (Estibb)</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>• [T-06] Im²plem²entación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
-• [T-07] Maquetación de vista de Login con estáilos estilos CSS nativos y validíación de cam²pos. (Estibb)</t>
+          <t>• [T-06] Implementación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
+• [T-07] Maquetación de vista de Login con estilos estilos CSS nativos y validación de campos. (Estibb)</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>• [T-03] Entorno Docker local com²pletam²ente operativo para todo el equipo. (Gerardo)
-• [T-04] Esquem²a relacional de tablas de Usuarios y Roles aplicado en PostgreSQL Docker local. (Diego)
-• [T-05] Estructura visual de com²ponentes de Login aprobadía por el equipo. (Estibb)</t>
+          <t>• [T-03] Entorno Docker local completamente operativo para todo el equipo. (Gerardo)
+• [T-04] Esquema relacional de tablas de Usuarios y Roles aplicado en PostgreSQL Docker local. (Diego)
+• [T-05] Estructura visual de componentes de Login aprobada por el equipo. (Estibb)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 — Día 4
+          <t>Sprint 1 —— Día 4
 (Jueves 17/09/2026)</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>• [T-10] Pruebas unitarias de endpoints de autenticación con pytestá. (Diego)
-• [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas autom²atizadías locales. (Gerardo)
-• [T-12] Pruebas unitarias de com²ponentes en Angular con Jasm²ine/Karm²a. (Estibb)</t>
+          <t>• [T-10] Pruebas unitarias de endpoints de autenticación con pytest. (Diego)
+• [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas automatizadías locales. (Gerardo)
+• [T-12] Pruebas unitarias de componentes en Angular con Jasmine/Karma. (Estibb)</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Sin bloqueos (Im²pedim²ento de T-07 resuelto con la publicación del endpoint de login).</t>
+          <t>Sin bloqueos (Impedimento de T-07 resuelto con la publicación del endpoint de login).</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>• [T-07] Integración del form²ulario de Login con API REST y gestáión de tokens JWT en LocalStorage. (Estibb)
-• [T-08] Param²etrización de catálogo de insum²os y fórm²ulas de consum²o por m²² (HU-02). (Diego)
+          <t>• [T-07] Integración del formulario de Login con API REST y gestión de tokens JWT en LocalStorage. (Estibb)
+• [T-08] Parametrización de catálogo de insumos y fórmulas de consumo por m² (HU-02). (Diego)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)</t>
         </is>
       </c>
@@ -1008,32 +1008,32 @@
     <row r="10" ht="70" customHeight="1">
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 — Día 5
+          <t>Sprint 1 —— Día 5
 (Viernes 18/09/2026)</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>• [T-13] Pruebas de integración de servicios y validíación de contenedores Docker en desarrollo local. (Gerardo)
-• [T-14] Dem²ostración funcional interna del increm²ento de software (Sprint Review interna). (Equipo)</t>
+          <t>• [T-13] Pruebas de integración de servicios y validación de contenedores Docker en desarrollo local. (Gerardo)
+• [T-14] Demostración funcional interna del incremento de software (Sprint Review interna). (Equipo)</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>Sin im²pedim²entos.</t>
+          <t>Sin impedimentos.</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>• [T-10] Pruebas unitarias de endpoints con pytestá y verificación de cobertura de código. (Diego)
+          <t>• [T-10] Pruebas unitarias de endpoints con pytest y verificación de cobertura de código. (Diego)
 • [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas de integración. (Gerardo)
-• [T-12] Pruebas unitarias de com²ponentes en Angular con Jasm²ine/Karm²a. (Estibb)</t>
+• [T-12] Pruebas unitarias de componentes en Angular con Jasmine/Karma. (Estibb)</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>• [T-07] Com²ponente de Login interactivo en Angular 21 consum²iendo API REST con ééxito. (Estibb)
-• [T-08] Param²etrización de recetas de insum²os por m²² (vinilo, lona, tinta) culm²inadía en PostgreSQL. (Diego)
+          <t>• [T-07] Componente de Login interactivo en Angular 21 consumiendo API REST con ééxito. (Estibb)
+• [T-08] Parametrización de recetas de insumos por m² (vinilo, lona, tinta) culminada en PostgreSQL. (Diego)
 • [T-09] Guards de navegación por roles activos en Angular 21 (bloqueo efectivo a no autorizados). (Estibb)</t>
         </is>
       </c>
@@ -1041,23 +1041,23 @@
     <row r="11" ht="185" customHeight="1">
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 — Día 6
+          <t>Sprint 1 —— Día 6
 (Sábado 19/09/2026)</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>• [T-15] Backlog Refinem²ent y preparación de tareas para Sprint 2 (Cotizador y Talonario Digital HU-03, HU-04). (Equipo)</t>
+          <t>• [T-15] Backlog Refinement y preparación de tareas para Sprint 2 (Cotizador y Talonario Digital HU-03, HU-04). (Equipo)</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Cero im²pedim²entos al cierre de la sem²ana (Despliegue a servidor VPS particular planificado para sem²ana 11).</t>
+          <t>Cero impedimentos al cierre de la semana (Despliegue a servidor VPS particular planificado para semana 11).</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>• [T-14] Dem²ostración funcional interna del increm²ento y verificación de Definition of Done (DoD). (Gerardo, Estibb, Diego)</t>
+          <t>• [T-14] Demostración funcional interna del incremento y verificación de Definition of Done (DoD). (Gerardo, Estibb, Diego)</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
@@ -1069,12 +1069,12 @@
 • [T-05] Maquetación de interfaz de Login en Angular 21. (Estibb)
 • [T-06] API de Autenticación JWT en FastAPI. (Diego)
 • [T-07] Login frontend interactivo en Angular 21. (Estibb)
-• [T-08] Recetas de insum²os por m²² param²etrizadías en PostgreSQL. (Diego)
+• [T-08] Recetas de insumos por m² parametrizadías en PostgreSQL. (Diego)
 • [T-09] Guards de navegación RBAC en Angular 21. (Estibb)
-• [T-10] Suite de pruebas unitarias pytestá (cobertura 84%). (Diego)
+• [T-10] Suite de pruebas unitarias pytest (cobertura 84%). (Diego)
 • [T-11] Pipeline CI/CD en GitHub Actions para pruebas locales. (Gerardo)
-• [T-12] Pruebas unitarias frontend con Jasm²ine/Karm²a. (Estibb)
-• [T-13] Integración com²pleta de servicios locales y verificación en Docker. (Gerardo)</t>
+• [T-12] Pruebas unitarias frontend con Jasmine/Karma. (Estibb)
+• [T-13] Integración completa de servicios locales y verificación en Docker. (Gerardo)</t>
         </is>
       </c>
     </row>
@@ -1101,9 +1101,9 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Im²pedim²entos: 1 registrado (T-07)
-Estado de im²pedim²entos: 100% resuelto
-Despliegue: Sin despliegue (VPS en sem²ana 11)</t>
+          <t>Impedimentos: 1 registrado (T-07)
+Estado de impedimentos: 100% resuelto
+Despliegue: Sin despliegue (VPS en semana 11)</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
@@ -1115,10 +1115,10 @@
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>Com²pletadías al 100%: 13 tareas
+          <t>Completadías al 100%: 13 tareas
 Porcentaje de Ééxito de Sprint 1: 86.7%
-Story Points com²pletados: 8 SP
-Estado: Conform²e para Sprint Review</t>
+Story Points completados: 8 SP
+Estado: Conforme para Sprint Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sem04): reestructurar scrum diario sincerando tareas de desarrollo lun-vie, sprint review y traspaso a sprint 2
</commit_message>
<xml_diff>
--- a/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
+++ b/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
@@ -795,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="B2:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -807,7 +807,6 @@
     <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="9" t="inlineStr">
         <is>
@@ -875,7 +874,7 @@
     <row r="6" ht="94" customHeight="1">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 —— Día 1
+          <t>Sprint 1 — Día 1
 (Lunes 14/09/2026)</t>
         </is>
       </c>
@@ -883,10 +882,8 @@
         <is>
           <t>• [T-03] Configuración de Docker Compose para entorno local (Angular 21 + FastAPI + PostgreSQL nativo). (Gerardo)
 • [T-04] Modelamiento de tablas relacionales de Usuarios y Roles en PostgreSQL Docker. (Diego)
-• [T-05] Maquetación inicial de estructura HTML/CSS de Login y formulario reactivo en Angular 21. (Estibb)
-• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
-• [T-07] Maquetación de componente de Login y validaciones de interfaz en Angular 21. (Estibb)
-• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)</t>
+• [T-05] Maquetación inicial de estructura HTML/CSS de Login en Angular 21. (Estibb)
+• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)</t>
         </is>
       </c>
       <c r="D6" s="17" t="inlineStr">
@@ -902,23 +899,24 @@
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>Fase de inicio de iteración: Tareas 01 y 02 en proceso de arranque.</t>
+          <t>• [T-01] Sprint Planning 1: Desglose formalizado en el Product Backlog y Sprint Backlog. (Equipo)
+• [T-02] Repositorio GitHub inicializado con estructura de ramas. (Gerardo)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 —— Día 2
+          <t>Sprint 1 — Día 2
 (Martes 15/09/2026)</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
-• [T-07] Maquetación de componente de Login y validaciones en Angular 21. (Estibb)
-• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)
-• [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)</t>
+          <t>• [T-05] Maquetación de interfaz y formulario reactivo de Login en Angular 21. (Estibb)
+• [T-06] Implementación de servicio de autenticación JWT y hashing bcrypt en FastAPI. (Diego)
+• [T-07] Integración del formulario de Login con API REST. (Estibb)
+• [T-08] Modelamiento relacional de tablas de Insumos y Recetas por m² en PostgreSQL Docker. (Diego)</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
@@ -929,29 +927,28 @@
       <c r="E7" s="18" t="inlineStr">
         <is>
           <t>• [T-03] Configuración de Docker Compose para entorno local unificado (FastAPI, PostgreSQL, Angular). (Gerardo)
-• [T-04] Modelamiento y creación de tablas relacionales de Usuarios y Roles en PostgreSQL. (Diego)
-• [T-05] Maquetación inicial de estructura HTML/CSS de Login en Angular 21. (Estibb)</t>
+• [T-04] Modelamiento y creación de tablas relacionales de Usuarios y Roles en PostgreSQL Docker. (Diego)</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>• [T-01] Sprint Planning 1: Desglose de HU-01 y HU-02 formalizado en el Product Backlog. (Equipo)
-• [T-02] Repositorio GitHub configurado con reglas de protección de rama main. (Gerardo)</t>
+          <t>• [T-03] Entorno Docker Compose local completamente operativo para todo el equipo. (Gerardo)
+• [T-04] Esquema relacional de tablas de Usuarios y Roles aplicado en PostgreSQL Docker. (Diego)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 —— Día 3
+          <t>Sprint 1 — Día 3
 (Miércoles 16/09/2026)</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>• [T-08] Parametrización de catálogo de insumos y recetas por m² en base de datos PostgreSQL. (Diego)
+          <t>• [T-07] Integración del formulario de Login con API REST y gestión de sesión JWT. (Estibb)
 • [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)
-• [T-10] Pruebas unitarias de endpoints de autenticación con pytest. (Diego)</t>
+• [T-10] Pruebas unitarias de endpoints de autenticación con pytest en backend. (Diego)</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
@@ -961,30 +958,29 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>• [T-06] Implementación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
-• [T-07] Maquetación de vista de Login con estilos estilos CSS nativos y validación de campos. (Estibb)</t>
+          <t>• [T-05] Maquetación de vista de Login con estilos CSS nativos y validación de campos. (Estibb)
+• [T-06] Implementación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
+• [T-08] Modelamiento relacional de tablas de Insumos y Recetas por m² en PostgreSQL Docker. (Diego)</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>• [T-03] Entorno Docker local completamente operativo para todo el equipo. (Gerardo)
-• [T-04] Esquema relacional de tablas de Usuarios y Roles aplicado en PostgreSQL Docker local. (Diego)
-• [T-05] Estructura visual de componentes de Login aprobada por el equipo. (Estibb)</t>
+          <t>• [T-05] Estructura visual de componentes y formulario reactivo de Login aprobada. (Estibb)
+• [T-08] Tablas relacionales de Insumos y Recetas migradas en PostgreSQL Docker (base de HU-02). (Diego)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 —— Día 4
+          <t>Sprint 1 — Día 4
 (Jueves 17/09/2026)</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>• [T-10] Pruebas unitarias de endpoints de autenticación con pytest. (Diego)
-• [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas automatizadías locales. (Gerardo)
-• [T-12] Pruebas unitarias de componentes en Angular con Jasmine/Karma. (Estibb)</t>
+          <t>• [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)
+• [T-10] Pruebas unitarias de endpoints de autenticación con pytest en backend. (Diego)</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
@@ -994,87 +990,83 @@
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>• [T-07] Integración del formulario de Login con API REST y gestión de tokens JWT en LocalStorage. (Estibb)
-• [T-08] Parametrización de catálogo de insumos y fórmulas de consumo por m² (HU-02). (Diego)
-• [T-09] Creación de Angular AuthGuard para protección de rutas según rol (RBAC). (Estibb)</t>
+          <t>• [T-06] Culminación de endpoints de autenticación JWT y roles en FastAPI. (Diego)
+• [T-07] Integración del formulario de Login con API REST y almacenamiento seguro de token JWT. (Estibb)
+• [T-10] Pruebas unitarias de endpoints de autenticación con pytest en backend. (Diego)</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>• [T-06] Servicio de autenticación JWT y endpoints de login concluidos y verificados en Swagger UI. (Diego)</t>
+          <t>• [T-06] Servicio de autenticación JWT y endpoints de login concluidos en FastAPI. (Diego)
+• [T-07] Componente de Login interactivo en Angular 21 consumiendo API REST con éxito. (Estibb)
+• [T-10] Suite de pruebas unitarias pytest para autenticación y usuarios con 84% de cobertura. (Diego)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 —— Día 5
-(Viernes 18/09/2026)</t>
+          <t>Sprint 1 — Día 5
+(Viernes 18/09/2026)
+Cierre de Desarrollo</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>• [T-13] Pruebas de integración de servicios y validación de contenedores Docker en desarrollo local. (Gerardo)
-• [T-14] Demostración funcional interna del incremento de software (Sprint Review interna). (Equipo)</t>
+          <t>• Preparación de material de demostración funcional para la sesión de clase del sábado.
+• Registro de tareas técnicas en proceso y deuda técnica para traslado a Sprint 2.</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>Sin impedimentos.</t>
+          <t>Sin impedimentos. Entorno de desarrollo local validado para la presentación académica.</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>• [T-10] Pruebas unitarias de endpoints con pytest y verificación de cobertura de código. (Diego)
-• [T-11] Configuración de pipeline CI/CD en GitHub Actions para pruebas de integración. (Gerardo)
-• [T-12] Pruebas unitarias de componentes en Angular con Jasmine/Karma. (Estibb)</t>
+          <t>• [T-09] Implementación de Angular AuthGuard y restricción de navegación por roles RBAC. (Estibb)
+• Verificación técnica funcional interna en Docker local de los criterios de DoD para HU-01. (Equipo)</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>• [T-07] Componente de Login interactivo en Angular 21 consumiendo API REST con ééxito. (Estibb)
-• [T-08] Parametrización de recetas de insumos por m² (vinilo, lona, tinta) culminada en PostgreSQL. (Diego)
-• [T-09] Guards de navegación por roles activos en Angular 21 (bloqueo efectivo a no autorizados). (Estibb)</t>
+          <t>• [T-09] Guards de navegación por roles activos en Angular 21 (bloqueo efectivo a no autorizados). (Estibb)
+• Verificación técnica interna en Docker local completada con éxito. Cierre del ciclo de codificación de Sprint 1. (Equipo)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="185" customHeight="1">
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Sprint 1 —— Día 6
-(Sábado 19/09/2026)</t>
+          <t>Sprint 1 — Día 6
+(Sábado 19/09/2026)
+Sprint Review en Clase</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>• [T-15] Backlog Refinement y preparación de tareas para Sprint 2 (Cotizador y Talonario Digital HU-03, HU-04). (Equipo)</t>
+          <t>• [T-11] Parametrización de catálogo de insumos y recetas por m² en interfaz web (HU-02 para Sprint 2).
+• [T-12] Implementación de pruebas unitarias de componentes en Angular (Deuda técnica Sprint 2).
+• [T-13] Configuración de pipeline CI/CD en GitHub Actions (Deuda técnica Sprint 2).
+• [T-14] Refinamiento de Product Backlog para Sprint 2 (Cotizador y Talonario Digital HU-03, HU-04).</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Cero impedimentos al cierre de la semana (Despliegue a servidor VPS particular planificado para semana 11).</t>
+          <t>Cero impedimentos al cierre del Sprint 1. Tareas no críticas trasladadas planificadamente al Sprint 2.</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>• [T-14] Demostración funcional interna del incremento y verificación de Definition of Done (DoD). (Gerardo, Estibb, Diego)</t>
+          <t>• Presentación del incremento de software (HU-01) en sesión de clase con el docente y Product Owner.
+• Sprint Retrospective y traspaso formal de tareas técnicas al backlog del Sprint 2.</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>• [T-01] Sprint Planning 1. (Equipo)
-• [T-02] Repositorio Git y branching. (Gerardo)
-• [T-03] Entorno Docker local unificado (FastAPI + PostgreSQL + Angular). (Gerardo)
-• [T-04] Tablas relacionales en PostgreSQL nativo Docker. (Diego)
-• [T-05] Maquetación de interfaz de Login en Angular 21. (Estibb)
-• [T-06] API de Autenticación JWT en FastAPI. (Diego)
-• [T-07] Login frontend interactivo en Angular 21. (Estibb)
-• [T-08] Recetas de insumos por m² parametrizadías en PostgreSQL. (Diego)
-• [T-09] Guards de navegación RBAC en Angular 21. (Estibb)
-• [T-10] Suite de pruebas unitarias pytest (cobertura 84%). (Diego)
-• [T-11] Pipeline CI/CD en GitHub Actions para pruebas locales. (Gerardo)
-• [T-12] Pruebas unitarias frontend con Jasmine/Karma. (Estibb)
-• [T-13] Integración completa de servicios locales y verificación en Docker. (Gerardo)</t>
+          <t>• Incremento de software de autenticación y roles validado y presentado ante el docente en clase.
+• Cierre formal del Sprint 1 conforme a la Definition of Done para HU-01 (3 SP devengados).
+• Deuda técnica (CI/CD, pruebas de componentes y recetas en interfaz) programada para Sprint 2.</t>
         </is>
       </c>
     </row>
@@ -1094,8 +1086,8 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>Total Planificadías: 15 tareas técnicas
-Historias cubiertas: HU-01 y base HU-02
+          <t>Total Planificadas: 14 tareas técnicas
+Historias cubiertas: HU-01 (100%) y HU-02 (base DB)
 Entorno: 100% Desarrollo Local en Docker</t>
         </is>
       </c>
@@ -1108,17 +1100,19 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>En ejecución: 1 tarea (T-14 revisión DoD)
-Avance funcional: Dentro del plazo
-Pruebas unitarias: 84% cobertura</t>
+          <t>Tareas trasladadas a Sprint 2: 4 tareas
+• Interfaz de recetas por m² (HU-02)
+• Pruebas unitarias Angular (deuda)
+• Pipeline CI/CD GitHub Actions (deuda)
+• Refinamiento Sprint 2 (Cotizador)</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>Completadías al 100%: 13 tareas
-Porcentaje de Ééxito de Sprint 1: 86.7%
-Story Points completados: 8 SP
-Estado: Conforme para Sprint Review</t>
+          <t>Completadas en desarrollo: 10 tareas
+Porcentaje de avance técnico: 71.4%
+Story Points devengados: 3 SP (HU-01)
+Estado: Conforme en Sprint Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sem04-05): subsanar observaciones docentes de semana 4 y generar acta de aceptacion formal
</commit_message>
<xml_diff>
--- a/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
+++ b/docs/entregables/SEM04/SCRUM_DIARIO.xlsx
@@ -958,14 +958,14 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>• [T-05] Maquetación de vista de Login con estilos CSS nativos y validación de campos. (Estibb)
+          <t>• [T-05] Maquetación de vista de Login con estilos CSS nativos, validación de campos y diseño responsive. (Estibb)
 • [T-06] Implementación de servicio de autenticación JWT y endpoints de login en FastAPI. (Diego)
 • [T-08] Modelamiento relacional de tablas de Insumos y Recetas por m² en PostgreSQL Docker. (Diego)</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>• [T-05] Estructura visual de componentes y formulario reactivo de Login aprobada. (Estibb)
+          <t>• [T-05] Maquetación de interfaz y componentes visuales de Login aprobada técnicamente. (Estibb)
 • [T-08] Tablas relacionales de Insumos y Recetas migradas en PostgreSQL Docker (base de HU-02). (Diego)</t>
         </is>
       </c>
@@ -990,15 +990,16 @@
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>• [T-06] Culminación de endpoints de autenticación JWT y roles en FastAPI. (Diego)
-• [T-07] Integración del formulario de Login con API REST y almacenamiento seguro de token JWT. (Estibb)
+          <t>• [T-05/T-07] Integración completa de la maquetación de Login con el servicio de autenticación REST en Angular 21. (Estibb)
+• [T-06] Culminación de endpoints de autenticación JWT y roles en FastAPI. (Diego)
 • [T-10] Pruebas unitarias de endpoints de autenticación con pytest en backend. (Diego)</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>• [T-06] Servicio de autenticación JWT y endpoints de login concluidos en FastAPI. (Diego)
-• [T-07] Componente de Login interactivo en Angular 21 consumiendo API REST con éxito. (Estibb)
+          <t>• [T-05] Maquetación responsive de Login y Shell base: 100% CULMINADA E INTEGRADA A HECHO (Done) en Angular 21. (Estibb)
+• [T-06] Servicio de autenticación JWT y endpoints de login concluidos en FastAPI. (Diego)
+• [T-07] Componente interactivo de Login consumiendo API REST con almacenamiento seguro de token JWT en HECHO (Done). (Estibb)
 • [T-10] Suite de pruebas unitarias pytest para autenticación y usuarios con 84% de cobertura. (Diego)</t>
         </is>
       </c>
@@ -1025,12 +1026,12 @@
       <c r="E10" s="18" t="inlineStr">
         <is>
           <t>• [T-09] Implementación de Angular AuthGuard y restricción de navegación por roles RBAC. (Estibb)
-• Verificación técnica funcional interna en Docker local de los criterios de DoD para HU-01. (Equipo)</t>
+• Verificación técnica funcional interna en Docker local de los criterios de DoD para HU-01 (Maquetación + API + Roles). (Equipo)</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>• [T-09] Guards de navegación por roles activos en Angular 21 (bloqueo efectivo a no autorizados). (Estibb)
+          <t>• [T-05/T-09] Maquetación responsive y Guards de navegación por rol plenamente operativos e integrados en HECHO (Done). (Estibb)
 • Verificación técnica interna en Docker local completada con éxito. Cierre del ciclo de codificación de Sprint 1. (Equipo)</t>
         </is>
       </c>
@@ -1058,14 +1059,14 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>• Presentación del incremento de software (HU-01) en sesión de clase con el docente y Product Owner.
+          <t>• Presentación del incremento de software funcional (HU-01: Maquetación, Auth y Roles) en sesión de clase ante el docente.
 • Sprint Retrospective y traspaso formal de tareas técnicas al backlog del Sprint 2.</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>• Incremento de software de autenticación y roles validado y presentado ante el docente en clase.
-• Cierre formal del Sprint 1 conforme a la Definition of Done para HU-01 (3 SP devengados).
+          <t>• Incremento de software de autenticación, maquetación y roles validado y presentado ante el docente en clase.
+• Cierre formal del ciclo de desarrollo conforme a la Definition of Done para HU-01 (3 SP devengados).
 • Deuda técnica (CI/CD, pruebas de componentes y recetas en interfaz) programada para Sprint 2.</t>
         </is>
       </c>
@@ -1109,8 +1110,18 @@
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>Completadas en desarrollo: 10 tareas
-Porcentaje de avance técnico: 71.4%
+          <t>Completadas en desarrollo (HECHO / Done): 10 tareas
+• [T-01] Sprint Planning 1 y Backlog
+• [T-02] Repositorio Git y ramas
+• [T-03] Docker Compose local unificado
+• [T-04] Tablas relacionales de Usuarios y Roles
+• [T-05] Maquetación de interfaz Login y Shell (HECHO)
+• [T-06] API Auth JWT y bcrypt en FastAPI
+• [T-07] Integración Login con API REST (HECHO)
+• [T-08] Modelo de tablas de Insumos en DB
+• [T-09] Guards de navegación por rol RBAC
+• [T-10] Pruebas unitarias backend (pytest)
+Porcentaje de avance técnico: 71.4% (10 de 14)
 Story Points devengados: 3 SP (HU-01)
 Estado: Conforme en Sprint Review</t>
         </is>

</xml_diff>